<commit_message>
PLTUR çözüldü: CFO = PDF satırı (filo alımları dahil), MDV = yatırım bölümü satırı, kira yok → 2026/06 FCF 1.317,6 (Evo 2.147,8); master ve P/FCF yenilendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012VyUPTEQJx1C4q1PKw5aha
</commit_message>
<xml_diff>
--- a/FCF_K13/PFCF_GETIRI.xlsx
+++ b/FCF_K13/PFCF_GETIRI.xlsx
@@ -35599,24 +35599,24 @@
         <v>3788.73</v>
       </c>
       <c r="I480" s="7" t="n">
-        <v>2147.827</v>
+        <v>1317.5914384</v>
       </c>
       <c r="J480" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K480" s="4" t="s">
-        <v>154</v>
+        <v>33</v>
       </c>
       <c r="L480" s="4" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="M480" s="8" t="n">
         <f aca="false">IF(OR(H480="",I480=""),"",IF(I480&gt;0,H480/I480,""))</f>
-        <v>1.76398285336761</v>
+        <v>2.87549682669523</v>
       </c>
       <c r="N480" s="4" t="str">
         <f aca="false">IF(I480="",IF(K480="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I480&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K480="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
-        <v>FCF KOŞULLU — yorum yapılmaz</v>
+        <v/>
       </c>
       <c r="O480" s="9" t="n">
         <f aca="false">IF(Q480="","",F480*R480/Q480-1)</f>

</xml_diff>

<commit_message>
Sistematik Evo hatası kontrolü: 75 şirket/226 dönem belgeden (120 teyit, 73 düzeltme); BRLSM/VANGD çözüldü; master, P/FCF, diff-set güncellendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012VyUPTEQJx1C4q1PKw5aha
</commit_message>
<xml_diff>
--- a/FCF_K13/PFCF_GETIRI.xlsx
+++ b/FCF_K13/PFCF_GETIRI.xlsx
@@ -5142,7 +5142,7 @@
         <v>6403.32</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>-406.025</v>
+        <v>-406.0259744</v>
       </c>
       <c r="J9" s="4" t="s">
         <v>32</v>
@@ -5151,7 +5151,7 @@
         <v>33</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M9" s="8" t="str">
         <f aca="false">IF(OR(H9="",I9=""),"",IF(I9&gt;0,H9/I9,""))</f>
@@ -9330,7 +9330,7 @@
         <v>9150</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>-0.0900000000000105</v>
+        <v>-0.0903120000000044</v>
       </c>
       <c r="J75" s="4" t="s">
         <v>32</v>
@@ -9339,7 +9339,7 @@
         <v>33</v>
       </c>
       <c r="L75" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M75" s="8" t="str">
         <f aca="false">IF(OR(H75="",I75=""),"",IF(I75&gt;0,H75/I75,""))</f>
@@ -9464,20 +9464,20 @@
         <v>7187.25</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>1752.834604</v>
+        <v>1752.8383072</v>
       </c>
       <c r="J77" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K77" s="4" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
       <c r="L77" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M77" s="8" t="n">
         <f aca="false">IF(OR(H77="",I77=""),"",IF(I77&gt;0,H77/I77,""))</f>
-        <v>4.10035834732984</v>
+        <v>4.10034968455304</v>
       </c>
       <c r="N77" s="4" t="str">
         <f aca="false">IF(I77="",IF(K77="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I77&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K77="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -13097,7 +13097,7 @@
         <v>2705.32</v>
       </c>
       <c r="I132" s="7" t="n">
-        <v>-351.893</v>
+        <v>-351.8936208</v>
       </c>
       <c r="J132" s="4" t="s">
         <v>32</v>
@@ -13106,7 +13106,7 @@
         <v>33</v>
       </c>
       <c r="L132" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M132" s="8" t="str">
         <f aca="false">IF(OR(H132="",I132=""),"",IF(I132&gt;0,H132/I132,""))</f>
@@ -13499,16 +13499,16 @@
         <v>11356.81977738</v>
       </c>
       <c r="I138" s="7" t="n">
-        <v>-563.771</v>
+        <v>-563.7706496</v>
       </c>
       <c r="J138" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K138" s="4" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
       <c r="L138" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M138" s="8" t="str">
         <f aca="false">IF(OR(H138="",I138=""),"",IF(I138&gt;0,H138/I138,""))</f>
@@ -15609,20 +15609,20 @@
         <v>1553.8</v>
       </c>
       <c r="I170" s="7" t="n">
-        <v>1036.616</v>
+        <v>1036.6163248</v>
       </c>
       <c r="J170" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K170" s="4" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
       <c r="L170" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M170" s="8" t="n">
         <f aca="false">IF(OR(H170="",I170=""),"",IF(I170&gt;0,H170/I170,""))</f>
-        <v>1.49891570263241</v>
+        <v>1.49891523298148</v>
       </c>
       <c r="N170" s="4" t="str">
         <f aca="false">IF(I170="",IF(K170="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I170&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K170="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -16001,7 +16001,7 @@
         <v>1254.375</v>
       </c>
       <c r="I176" s="7" t="n">
-        <v>-132.539</v>
+        <v>-132.5397248</v>
       </c>
       <c r="J176" s="4" t="s">
         <v>32</v>
@@ -16010,7 +16010,7 @@
         <v>33</v>
       </c>
       <c r="L176" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M176" s="8" t="str">
         <f aca="false">IF(OR(H176="",I176=""),"",IF(I176&gt;0,H176/I176,""))</f>
@@ -16592,7 +16592,7 @@
         <v>3108</v>
       </c>
       <c r="I185" s="7" t="n">
-        <v>645.578</v>
+        <v>645.5777056</v>
       </c>
       <c r="J185" s="4" t="s">
         <v>32</v>
@@ -16601,11 +16601,11 @@
         <v>33</v>
       </c>
       <c r="L185" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M185" s="8" t="n">
         <f aca="false">IF(OR(H185="",I185=""),"",IF(I185&gt;0,H185/I185,""))</f>
-        <v>4.81429044979848</v>
+        <v>4.81429264523846</v>
       </c>
       <c r="N185" s="4" t="str">
         <f aca="false">IF(I185="",IF(K185="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I185&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K185="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -17807,16 +17807,16 @@
         <v>3841.6</v>
       </c>
       <c r="I204" s="7" t="n">
-        <v>-840.062</v>
+        <v>-840.0628896</v>
       </c>
       <c r="J204" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K204" s="4" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
       <c r="L204" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M204" s="8" t="str">
         <f aca="false">IF(OR(H204="",I204=""),"",IF(I204&gt;0,H204/I204,""))</f>
@@ -17941,7 +17941,7 @@
         <v>2604.96</v>
       </c>
       <c r="I206" s="7" t="n">
-        <v>-172.025</v>
+        <v>-172.025048</v>
       </c>
       <c r="J206" s="4" t="s">
         <v>32</v>
@@ -17950,7 +17950,7 @@
         <v>33</v>
       </c>
       <c r="L206" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M206" s="8" t="str">
         <f aca="false">IF(OR(H206="",I206=""),"",IF(I206&gt;0,H206/I206,""))</f>
@@ -19133,7 +19133,7 @@
         <v>4641</v>
       </c>
       <c r="I224" s="7" t="n">
-        <v>507.641</v>
+        <v>507.6426352</v>
       </c>
       <c r="J224" s="4" t="s">
         <v>32</v>
@@ -19142,11 +19142,11 @@
         <v>33</v>
       </c>
       <c r="L224" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M224" s="8" t="n">
         <f aca="false">IF(OR(H224="",I224=""),"",IF(I224&gt;0,H224/I224,""))</f>
-        <v>9.14228756148538</v>
+        <v>9.14225811268108</v>
       </c>
       <c r="N224" s="4" t="str">
         <f aca="false">IF(I224="",IF(K224="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I224&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K224="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -22191,7 +22191,7 @@
         <v>137775</v>
       </c>
       <c r="I272" s="7" t="n">
-        <v>11617.73</v>
+        <v>11617.7373744</v>
       </c>
       <c r="J272" s="4" t="s">
         <v>32</v>
@@ -22200,11 +22200,11 @@
         <v>33</v>
       </c>
       <c r="L272" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M272" s="8" t="n">
         <f aca="false">IF(OR(H272="",I272=""),"",IF(I272&gt;0,H272/I272,""))</f>
-        <v>11.8590292595886</v>
+        <v>11.8590217320277</v>
       </c>
       <c r="N272" s="4" t="str">
         <f aca="false">IF(I272="",IF(K272="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I272&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K272="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -22392,7 +22392,7 @@
         <v>1992.9</v>
       </c>
       <c r="I275" s="7" t="n">
-        <v>-582.559</v>
+        <v>-582.558512</v>
       </c>
       <c r="J275" s="4" t="s">
         <v>32</v>
@@ -22401,7 +22401,7 @@
         <v>33</v>
       </c>
       <c r="L275" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M275" s="8" t="str">
         <f aca="false">IF(OR(H275="",I275=""),"",IF(I275&gt;0,H275/I275,""))</f>
@@ -22949,7 +22949,7 @@
         <v>4003.19283616</v>
       </c>
       <c r="I284" s="7" t="n">
-        <v>-771.952</v>
+        <v>-771.953312</v>
       </c>
       <c r="J284" s="4" t="s">
         <v>32</v>
@@ -22958,7 +22958,7 @@
         <v>33</v>
       </c>
       <c r="L284" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M284" s="8" t="str">
         <f aca="false">IF(OR(H284="",I284=""),"",IF(I284&gt;0,H284/I284,""))</f>
@@ -25366,7 +25366,7 @@
         <v>9579.5</v>
       </c>
       <c r="I323" s="7" t="n">
-        <v>504.076</v>
+        <v>504.07848</v>
       </c>
       <c r="J323" s="4" t="s">
         <v>32</v>
@@ -25375,11 +25375,11 @@
         <v>33</v>
       </c>
       <c r="L323" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M323" s="8" t="n">
         <f aca="false">IF(OR(H323="",I323=""),"",IF(I323&gt;0,H323/I323,""))</f>
-        <v>19.0040787500298</v>
+        <v>19.0039852524551</v>
       </c>
       <c r="N323" s="4" t="str">
         <f aca="false">IF(I323="",IF(K323="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I323&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K323="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -25567,7 +25567,7 @@
         <v>10095</v>
       </c>
       <c r="I326" s="7" t="n">
-        <v>915.675</v>
+        <v>915.6774576</v>
       </c>
       <c r="J326" s="4" t="s">
         <v>32</v>
@@ -25576,11 +25576,11 @@
         <v>33</v>
       </c>
       <c r="L326" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M326" s="8" t="n">
         <f aca="false">IF(OR(H326="",I326=""),"",IF(I326&gt;0,H326/I326,""))</f>
-        <v>11.0246539438119</v>
+        <v>11.0246243545834</v>
       </c>
       <c r="N326" s="4" t="str">
         <f aca="false">IF(I326="",IF(K326="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I326&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K326="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -26034,16 +26034,16 @@
         <v>3294.4725</v>
       </c>
       <c r="I333" s="7" t="n">
-        <v>-767.427</v>
+        <v>-767.4290128</v>
       </c>
       <c r="J333" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K333" s="4" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
       <c r="L333" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M333" s="8" t="str">
         <f aca="false">IF(OR(H333="",I333=""),"",IF(I333&gt;0,H333/I333,""))</f>
@@ -26434,7 +26434,7 @@
         <v>4708.04064</v>
       </c>
       <c r="I339" s="7" t="n">
-        <v>-177.866</v>
+        <v>-177.8681952</v>
       </c>
       <c r="J339" s="4" t="s">
         <v>32</v>
@@ -26443,7 +26443,7 @@
         <v>33</v>
       </c>
       <c r="L339" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M339" s="8" t="str">
         <f aca="false">IF(OR(H339="",I339=""),"",IF(I339&gt;0,H339/I339,""))</f>
@@ -29869,7 +29869,7 @@
         <v>24219.5</v>
       </c>
       <c r="I392" s="7" t="n">
-        <v>93.4279999999999</v>
+        <v>93.4278944</v>
       </c>
       <c r="J392" s="4" t="s">
         <v>32</v>
@@ -29878,11 +29878,11 @@
         <v>33</v>
       </c>
       <c r="L392" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M392" s="8" t="n">
         <f aca="false">IF(OR(H392="",I392=""),"",IF(I392&gt;0,H392/I392,""))</f>
-        <v>259.231707839192</v>
+        <v>259.232000844493</v>
       </c>
       <c r="N392" s="4" t="str">
         <f aca="false">IF(I392="",IF(K392="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I392&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K392="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -30662,7 +30662,7 @@
         <v>33</v>
       </c>
       <c r="L404" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M404" s="8" t="str">
         <f aca="false">IF(OR(H404="",I404=""),"",IF(I404&gt;0,H404/I404,""))</f>
@@ -32093,7 +32093,7 @@
         <v>2273.31</v>
       </c>
       <c r="I426" s="7" t="n">
-        <v>-153.87</v>
+        <v>-181.2489728</v>
       </c>
       <c r="J426" s="4" t="s">
         <v>32</v>
@@ -32102,7 +32102,7 @@
         <v>33</v>
       </c>
       <c r="L426" s="4" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="M426" s="8" t="str">
         <f aca="false">IF(OR(H426="",I426=""),"",IF(I426&gt;0,H426/I426,""))</f>
@@ -32867,7 +32867,7 @@
         <v>12973.15279854</v>
       </c>
       <c r="I438" s="7" t="n">
-        <v>-1015.45</v>
+        <v>-1015.4494096</v>
       </c>
       <c r="J438" s="4" t="s">
         <v>32</v>
@@ -32876,7 +32876,7 @@
         <v>33</v>
       </c>
       <c r="L438" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M438" s="8" t="str">
         <f aca="false">IF(OR(H438="",I438=""),"",IF(I438&gt;0,H438/I438,""))</f>
@@ -33984,7 +33984,7 @@
         <v>573.75</v>
       </c>
       <c r="I455" s="7" t="n">
-        <v>-103.035</v>
+        <v>-103.0356896</v>
       </c>
       <c r="J455" s="4" t="s">
         <v>32</v>
@@ -33993,7 +33993,7 @@
         <v>33</v>
       </c>
       <c r="L455" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M455" s="8" t="str">
         <f aca="false">IF(OR(H455="",I455=""),"",IF(I455&gt;0,H455/I455,""))</f>
@@ -35398,7 +35398,7 @@
         <v>2518.7927875</v>
       </c>
       <c r="I477" s="7" t="n">
-        <v>200.312</v>
+        <v>200.3121024</v>
       </c>
       <c r="J477" s="4" t="s">
         <v>32</v>
@@ -35407,11 +35407,11 @@
         <v>33</v>
       </c>
       <c r="L477" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M477" s="8" t="n">
         <f aca="false">IF(OR(H477="",I477=""),"",IF(I477&gt;0,H477/I477,""))</f>
-        <v>12.5743479546907</v>
+        <v>12.5743415266556</v>
       </c>
       <c r="N477" s="4" t="str">
         <f aca="false">IF(I477="",IF(K477="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I477&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K477="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -35465,7 +35465,7 @@
         <v>2138.5</v>
       </c>
       <c r="I478" s="7" t="n">
-        <v>121.425</v>
+        <v>121.424712</v>
       </c>
       <c r="J478" s="4" t="s">
         <v>32</v>
@@ -35474,11 +35474,11 @@
         <v>33</v>
       </c>
       <c r="L478" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M478" s="8" t="n">
         <f aca="false">IF(OR(H478="",I478=""),"",IF(I478&gt;0,H478/I478,""))</f>
-        <v>17.6116944616018</v>
+        <v>17.6117362337248</v>
       </c>
       <c r="N478" s="4" t="str">
         <f aca="false">IF(I478="",IF(K478="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I478&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K478="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -35532,7 +35532,7 @@
         <v>2478.36672</v>
       </c>
       <c r="I479" s="7" t="n">
-        <v>9.60300000000001</v>
+        <v>9.60355520000002</v>
       </c>
       <c r="J479" s="4" t="s">
         <v>32</v>
@@ -35541,11 +35541,11 @@
         <v>33</v>
       </c>
       <c r="L479" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M479" s="8" t="n">
         <f aca="false">IF(OR(H479="",I479=""),"",IF(I479&gt;0,H479/I479,""))</f>
-        <v>258.082549203374</v>
+        <v>258.067628954743</v>
       </c>
       <c r="N479" s="4" t="str">
         <f aca="false">IF(I479="",IF(K479="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I479&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K479="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -35800,7 +35800,7 @@
         <v>14062.59</v>
       </c>
       <c r="I483" s="7" t="n">
-        <v>169.909</v>
+        <v>169.9078768</v>
       </c>
       <c r="J483" s="4" t="s">
         <v>32</v>
@@ -35809,11 +35809,11 @@
         <v>33</v>
       </c>
       <c r="L483" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M483" s="8" t="n">
         <f aca="false">IF(OR(H483="",I483=""),"",IF(I483&gt;0,H483/I483,""))</f>
-        <v>82.7654214903272</v>
+        <v>82.7659686228273</v>
       </c>
       <c r="N483" s="4" t="str">
         <f aca="false">IF(I483="",IF(K483="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I483&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K483="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -38413,7 +38413,7 @@
         <v>602</v>
       </c>
       <c r="I524" s="7" t="n">
-        <v>74.11</v>
+        <v>74.1103312</v>
       </c>
       <c r="J524" s="4" t="s">
         <v>32</v>
@@ -38422,11 +38422,11 @@
         <v>33</v>
       </c>
       <c r="L524" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M524" s="8" t="n">
         <f aca="false">IF(OR(H524="",I524=""),"",IF(I524&gt;0,H524/I524,""))</f>
-        <v>8.12306031574686</v>
+        <v>8.12302401368839</v>
       </c>
       <c r="N524" s="4" t="str">
         <f aca="false">IF(I524="",IF(K524="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I524&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K524="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -38858,7 +38858,7 @@
         <v>518.08425</v>
       </c>
       <c r="I531" s="7" t="n">
-        <v>1.54299999999993</v>
+        <v>1.54268639999994</v>
       </c>
       <c r="J531" s="4" t="s">
         <v>32</v>
@@ -38867,11 +38867,11 @@
         <v>33</v>
       </c>
       <c r="L531" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M531" s="8" t="n">
         <f aca="false">IF(OR(H531="",I531=""),"",IF(I531&gt;0,H531/I531,""))</f>
-        <v>335.764257939095</v>
+        <v>335.832512686973</v>
       </c>
       <c r="N531" s="4" t="str">
         <f aca="false">IF(I531="",IF(K531="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I531&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K531="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -39104,7 +39104,7 @@
         <v>1368</v>
       </c>
       <c r="I535" s="7" t="n">
-        <v>324.29</v>
+        <v>320.3424768</v>
       </c>
       <c r="J535" s="4" t="s">
         <v>32</v>
@@ -39113,11 +39113,11 @@
         <v>33</v>
       </c>
       <c r="L535" s="4" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="M535" s="8" t="n">
         <f aca="false">IF(OR(H535="",I535=""),"",IF(I535&gt;0,H535/I535,""))</f>
-        <v>4.21844645224953</v>
+        <v>4.27042961540841</v>
       </c>
       <c r="N535" s="4" t="str">
         <f aca="false">IF(I535="",IF(K535="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I535&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K535="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -39171,7 +39171,7 @@
         <v>7191.6</v>
       </c>
       <c r="I536" s="7" t="n">
-        <v>554.258</v>
+        <v>554.2561824</v>
       </c>
       <c r="J536" s="4" t="s">
         <v>32</v>
@@ -39180,11 +39180,11 @@
         <v>33</v>
       </c>
       <c r="L536" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M536" s="8" t="n">
         <f aca="false">IF(OR(H536="",I536=""),"",IF(I536&gt;0,H536/I536,""))</f>
-        <v>12.9751848417163</v>
+        <v>12.9752273918885</v>
       </c>
       <c r="N536" s="4" t="str">
         <f aca="false">IF(I536="",IF(K536="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I536&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K536="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -40654,7 +40654,7 @@
         <v>1326</v>
       </c>
       <c r="I559" s="7" t="n">
-        <v>-94.143</v>
+        <v>-94.1420704</v>
       </c>
       <c r="J559" s="4" t="s">
         <v>32</v>
@@ -40663,7 +40663,7 @@
         <v>33</v>
       </c>
       <c r="L559" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M559" s="8" t="str">
         <f aca="false">IF(OR(H559="",I559=""),"",IF(I559&gt;0,H559/I559,""))</f>
@@ -41509,7 +41509,7 @@
         <v>138860.4</v>
       </c>
       <c r="I572" s="7" t="n">
-        <v>-880.248999999999</v>
+        <v>-880.2476432</v>
       </c>
       <c r="J572" s="4" t="s">
         <v>32</v>
@@ -41518,7 +41518,7 @@
         <v>33</v>
       </c>
       <c r="L572" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M572" s="8" t="str">
         <f aca="false">IF(OR(H572="",I572=""),"",IF(I572&gt;0,H572/I572,""))</f>
@@ -42208,7 +42208,7 @@
         <v>40301.93390625</v>
       </c>
       <c r="I583" s="7" t="n">
-        <v>2948.957</v>
+        <v>2948.9602752</v>
       </c>
       <c r="J583" s="4" t="s">
         <v>32</v>
@@ -42217,11 +42217,11 @@
         <v>33</v>
       </c>
       <c r="L583" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M583" s="8" t="n">
         <f aca="false">IF(OR(H583="",I583=""),"",IF(I583&gt;0,H583/I583,""))</f>
-        <v>13.6665044306343</v>
+        <v>13.6664892522219</v>
       </c>
       <c r="N583" s="4" t="str">
         <f aca="false">IF(I583="",IF(K583="NULL","FCF yok (NULL)","FCF kapsamı dışı"),IF(I583&lt;=0,"anlamsız (FCF ≤ 0)",IF(OR(K583="KOŞULLU"),"FCF KOŞULLU — yorum yapılmaz","")))</f>
@@ -43238,7 +43238,7 @@
         <v>1053.5</v>
       </c>
       <c r="I599" s="7" t="n">
-        <v>-2456.821</v>
+        <v>-2456.8216096</v>
       </c>
       <c r="J599" s="4" t="s">
         <v>32</v>
@@ -43247,7 +43247,7 @@
         <v>33</v>
       </c>
       <c r="L599" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M599" s="8" t="str">
         <f aca="false">IF(OR(H599="",I599=""),"",IF(I599&gt;0,H599/I599,""))</f>
@@ -43305,7 +43305,7 @@
         <v>1157.5985</v>
       </c>
       <c r="I600" s="7" t="n">
-        <v>-2.419</v>
+        <v>-2.4193344</v>
       </c>
       <c r="J600" s="4" t="s">
         <v>32</v>
@@ -43314,7 +43314,7 @@
         <v>33</v>
       </c>
       <c r="L600" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M600" s="8" t="str">
         <f aca="false">IF(OR(H600="",I600=""),"",IF(I600&gt;0,H600/I600,""))</f>
@@ -44167,7 +44167,7 @@
         <v>669.9</v>
       </c>
       <c r="I614" s="7" t="n">
-        <v>-536.127</v>
+        <v>-536.1262688</v>
       </c>
       <c r="J614" s="4" t="s">
         <v>32</v>
@@ -44176,7 +44176,7 @@
         <v>33</v>
       </c>
       <c r="L614" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M614" s="8" t="str">
         <f aca="false">IF(OR(H614="",I614=""),"",IF(I614&gt;0,H614/I614,""))</f>

</xml_diff>